<commit_message>
Publish polished BI case studies and verified project downloads
</commit_message>
<xml_diff>
--- a/files/Inventory_Health.xlsx
+++ b/files/Inventory_Health.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory dashboard" sheetId="1" r:id="Rba8ed916047e4f2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reorder analysis" sheetId="2" r:id="Rf3824a6f4c1d40a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item inputs" sheetId="3" r:id="Raaeabe0dd1394964"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory dashboard" sheetId="1" r:id="Rba198342db2b4c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reorder analysis" sheetId="2" r:id="Re1d7bcb876f2429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item inputs" sheetId="3" r:id="R2be9d2e4d9474664"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,13 +15,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="&quot;£&quot;#,##0"/>
     <x:numFmt numFmtId="201" formatCode="0.0&quot;x&quot;"/>
     <x:numFmt numFmtId="202" formatCode="&quot;£&quot;#,##0.00"/>
     <x:numFmt numFmtId="203" formatCode="0.0"/>
+    <x:numFmt numFmtId="204" formatCode="#,##0"/>
+    <x:numFmt numFmtId="205" formatCode="0.00&quot;x&quot;"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -43,8 +45,42 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF16384B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF16384B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="17"/>
+      <x:color rgb="FF16384B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF526575"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF087E83"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -61,6 +97,16 @@
         <x:fgColor rgb="FFFFF0BF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF16384B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF087E83"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -68,7 +114,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -82,6 +128,37 @@
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -93,7 +170,7 @@
         <x:color rgb="FF845000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0BF"/>
         </x:patternFill>
       </x:fill>
@@ -103,169 +180,217 @@
 </file>
 
 <file path=xl/drawings/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:r>
-              <a:rPr sz="1050">
-                <a:latin typeface="Arial"/>
-                <a:ea typeface="Arial"/>
-                <a:cs typeface="Arial"/>
-              </a:rPr>
-              <a:t>Stock and proposed orders by category (GBP)</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-      <c:txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr>
-            <a:defRPr sz="1050">
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:defRPr>
-          </a:pPr>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:plotArea>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Inventory value</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="325C80"/>
-            </a:solidFill>
-          </c:spPr>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Inventory dashboard'!$A$13:$A$16</c:f>
-              <c:strCache>
-                <c:ptCount val="0"/>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Inventory dashboard'!$B$13:$B$16</c:f>
-              <c:numCache>
-                <c:formatCode>"£"#,##0</c:formatCode>
-                <c:ptCount val="0"/>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Order cost</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="D39945"/>
-            </a:solidFill>
-          </c:spPr>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Inventory dashboard'!$A$13:$A$16</c:f>
-              <c:strCache>
-                <c:ptCount val="0"/>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Inventory dashboard'!$C$13:$C$16</c:f>
-              <c:numCache>
-                <c:formatCode>"£"#,##0</c:formatCode>
-                <c:ptCount val="0"/>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:axId val="48650112"/>
-        <c:axId val="48672768"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="48650112"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="48672768"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="48672768"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="£#,##0" sourceLinked="0"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:crossAx val="48650112"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-  </c:chart>
-  <c:spPr>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-      <a:solidFill>
-        <a:srgbClr val="D9D9D9"/>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-    </a:ln>
-  </c:spPr>
-</c:chartSpace>
+<ns0:chartSpace xmlns:ns0="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:ns1="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <ns0:lang val="en-US"/>
+  <ns0:roundedCorners val="0"/>
+  <ns0:chart>
+    <ns0:title>
+      <ns0:tx>
+        <ns0:rich>
+          <ns1:bodyPr/>
+          <ns1:lstStyle/>
+          <ns1:p>
+            <ns1:r>
+              <ns1:rPr sz="1050">
+                <ns1:latin typeface="Arial"/>
+                <ns1:ea typeface="Arial"/>
+                <ns1:cs typeface="Arial"/>
+              </ns1:rPr>
+              <ns1:t>Stock and proposed orders by category (GBP)</ns1:t>
+            </ns1:r>
+          </ns1:p>
+        </ns0:rich>
+      </ns0:tx>
+      <ns0:overlay val="0"/>
+      <ns0:txPr>
+        <ns1:bodyPr anchorCtr="1"/>
+        <ns1:lstStyle/>
+        <ns1:p>
+          <ns1:pPr>
+            <ns1:defRPr sz="1050">
+              <ns1:latin typeface="Arial"/>
+              <ns1:ea typeface="Arial"/>
+              <ns1:cs typeface="Arial"/>
+            </ns1:defRPr>
+          </ns1:pPr>
+        </ns1:p>
+      </ns0:txPr>
+    </ns0:title>
+    <ns0:plotArea>
+      <ns0:barChart>
+        <ns0:barDir val="col"/>
+        <ns0:varyColors val="0"/>
+        <ns0:ser>
+          <ns0:idx val="0"/>
+          <ns0:order val="0"/>
+          <ns0:tx>
+            <ns0:v>Inventory value</ns0:v>
+          </ns0:tx>
+          <ns0:spPr>
+            <ns1:solidFill>
+              <ns1:srgbClr val="325C80"/>
+            </ns1:solidFill>
+          </ns0:spPr>
+          <ns0:cat>
+            <ns0:strRef>
+              <ns0:f>'Inventory dashboard'!$A$13:$A$16</ns0:f>
+              <ns0:strCache>
+                <ns0:ptCount val="4"/>
+                <ns0:pt idx="0">
+                  <ns0:v>Sinks</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="1">
+                  <ns0:v>Taps</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="2">
+                  <ns0:v>Hoods</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="3">
+                  <ns0:v>Accessories</ns0:v>
+                </ns0:pt>
+              </ns0:strCache>
+            </ns0:strRef>
+          </ns0:cat>
+          <ns0:val>
+            <ns0:numRef>
+              <ns0:f>'Inventory dashboard'!$B$13:$B$16</ns0:f>
+              <ns0:numCache>
+                <ns0:formatCode>General</ns0:formatCode>
+                <ns0:ptCount val="4"/>
+                <ns0:pt idx="0">
+                  <ns0:v>637519.65</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="1">
+                  <ns0:v>482834.9600000001</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="2">
+                  <ns0:v>356572.66</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="3">
+                  <ns0:v>707090.2799999999</ns0:v>
+                </ns0:pt>
+              </ns0:numCache>
+            </ns0:numRef>
+          </ns0:val>
+        </ns0:ser>
+        <ns0:ser>
+          <ns0:idx val="1"/>
+          <ns0:order val="1"/>
+          <ns0:tx>
+            <ns0:v>Order cost</ns0:v>
+          </ns0:tx>
+          <ns0:spPr>
+            <ns1:solidFill>
+              <ns1:srgbClr val="D39945"/>
+            </ns1:solidFill>
+          </ns0:spPr>
+          <ns0:cat>
+            <ns0:strRef>
+              <ns0:f>'Inventory dashboard'!$A$13:$A$16</ns0:f>
+              <ns0:strCache>
+                <ns0:ptCount val="4"/>
+                <ns0:pt idx="0">
+                  <ns0:v>Sinks</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="1">
+                  <ns0:v>Taps</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="2">
+                  <ns0:v>Hoods</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="3">
+                  <ns0:v>Accessories</ns0:v>
+                </ns0:pt>
+              </ns0:strCache>
+            </ns0:strRef>
+          </ns0:cat>
+          <ns0:val>
+            <ns0:numRef>
+              <ns0:f>'Inventory dashboard'!$C$13:$C$16</ns0:f>
+              <ns0:numCache>
+                <ns0:formatCode>General</ns0:formatCode>
+                <ns0:ptCount val="4"/>
+                <ns0:pt idx="0">
+                  <ns0:v>290238.83</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="1">
+                  <ns0:v>87785.3</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="2">
+                  <ns0:v>168553.37</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="3">
+                  <ns0:v>220214.61000000002</ns0:v>
+                </ns0:pt>
+              </ns0:numCache>
+            </ns0:numRef>
+          </ns0:val>
+        </ns0:ser>
+        <ns0:axId val="48650112"/>
+        <ns0:axId val="48672768"/>
+      </ns0:barChart>
+      <ns0:catAx>
+        <ns0:axId val="48650112"/>
+        <ns0:scaling>
+          <ns0:orientation val="minMax"/>
+        </ns0:scaling>
+        <ns0:delete val="0"/>
+        <ns0:axPos val="b"/>
+        <ns0:majorGridlines>
+          <ns0:spPr>
+            <ns1:ln w="9525">
+              <ns1:solidFill>
+                <ns1:srgbClr val="CCCCCC"/>
+              </ns1:solidFill>
+              <ns1:prstDash val="dash"/>
+            </ns1:ln>
+          </ns0:spPr>
+        </ns0:majorGridlines>
+        <ns0:numFmt formatCode="General"/>
+        <ns0:majorTickMark val="none"/>
+        <ns0:minorTickMark val="none"/>
+        <ns0:tickLblPos val="nextTo"/>
+        <ns0:crossAx val="48672768"/>
+      </ns0:catAx>
+      <ns0:valAx>
+        <ns0:axId val="48672768"/>
+        <ns0:scaling>
+          <ns0:orientation val="minMax"/>
+        </ns0:scaling>
+        <ns0:delete val="0"/>
+        <ns0:axPos val="l"/>
+        <ns0:majorGridlines>
+          <ns0:spPr>
+            <ns1:ln w="9525">
+              <ns1:solidFill>
+                <ns1:srgbClr val="CCCCCC"/>
+              </ns1:solidFill>
+              <ns1:prstDash val="dash"/>
+            </ns1:ln>
+          </ns0:spPr>
+        </ns0:majorGridlines>
+        <ns0:numFmt formatCode="£#,##0" sourceLinked="0"/>
+        <ns0:majorTickMark val="none"/>
+        <ns0:minorTickMark val="none"/>
+        <ns0:crossAx val="48650112"/>
+        <ns0:crossBetween val="between"/>
+      </ns0:valAx>
+    </ns0:plotArea>
+    <ns0:legend>
+      <ns0:legendPos val="b"/>
+      <ns0:overlay val="0"/>
+    </ns0:legend>
+    <ns0:plotVisOnly val="1"/>
+  </ns0:chart>
+  <ns0:spPr>
+    <ns1:ln w="9525">
+      <ns1:solidFill>
+        <ns1:srgbClr val="D9D9D9"/>
+      </ns1:solidFill>
+      <ns1:prstDash val="solid"/>
+    </ns1:ln>
+  </ns0:spPr>
+</ns0:chartSpace>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -294,7 +419,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5889f2fc093d4fde"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re7bc14597163422c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -563,18 +688,18 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
-      <x:c r="A1" s="1"/>
-      <x:c r="B1" s="1"/>
-      <x:c r="C1" s="1"/>
-      <x:c r="D1" s="1"/>
-      <x:c r="E1" s="1"/>
-      <x:c r="F1" s="1"/>
-      <x:c r="G1" s="1"/>
-      <x:c r="H1" s="1"/>
-      <x:c r="I1" s="1"/>
-      <x:c r="J1" s="1"/>
-      <x:c r="K1" s="1"/>
-      <x:c r="L1" s="1"/>
+      <x:c r="A1" s="11"/>
+      <x:c r="B1" s="11"/>
+      <x:c r="C1" s="11"/>
+      <x:c r="D1" s="11"/>
+      <x:c r="E1" s="11"/>
+      <x:c r="F1" s="11"/>
+      <x:c r="G1" s="11"/>
+      <x:c r="H1" s="11"/>
+      <x:c r="I1" s="11"/>
+      <x:c r="J1" s="11"/>
+      <x:c r="K1" s="11"/>
+      <x:c r="L1" s="11"/>
       <x:c r="M1" s="1"/>
       <x:c r="N1" s="1"/>
       <x:c r="O1" s="1"/>
@@ -583,20 +708,20 @@
       <x:c r="R1" s="1"/>
     </x:row>
     <x:row r="2" ht="23" customHeight="1">
-      <x:c r="A2" s="2" t="str">
+      <x:c r="A2" s="16" t="str">
         <x:v>Inventory health and reorder analysis</x:v>
       </x:c>
-      <x:c r="B2" s="1"/>
-      <x:c r="C2" s="1"/>
-      <x:c r="D2" s="1"/>
-      <x:c r="E2" s="1"/>
-      <x:c r="F2" s="1"/>
-      <x:c r="G2" s="1"/>
-      <x:c r="H2" s="1"/>
-      <x:c r="I2" s="1"/>
-      <x:c r="J2" s="1"/>
-      <x:c r="K2" s="1"/>
-      <x:c r="L2" s="1"/>
+      <x:c r="B2" s="16"/>
+      <x:c r="C2" s="16"/>
+      <x:c r="D2" s="16"/>
+      <x:c r="E2" s="16"/>
+      <x:c r="F2" s="16"/>
+      <x:c r="G2" s="16"/>
+      <x:c r="H2" s="16"/>
+      <x:c r="I2" s="16"/>
+      <x:c r="J2" s="16"/>
+      <x:c r="K2" s="16"/>
+      <x:c r="L2" s="16"/>
       <x:c r="M2" s="1"/>
       <x:c r="N2" s="1"/>
       <x:c r="O2" s="1"/>
@@ -605,20 +730,20 @@
       <x:c r="R2" s="1"/>
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
-      <x:c r="A3" s="1" t="str">
+      <x:c r="A3" s="17" t="str">
         <x:v>Synthetic kitchen-products distributor. Snapshot: 21 Sep 2026. Currency: GBP.</x:v>
       </x:c>
-      <x:c r="B3" s="1"/>
-      <x:c r="C3" s="1"/>
-      <x:c r="D3" s="1"/>
-      <x:c r="E3" s="1"/>
-      <x:c r="F3" s="1"/>
-      <x:c r="G3" s="1"/>
-      <x:c r="H3" s="1"/>
-      <x:c r="I3" s="1"/>
-      <x:c r="J3" s="1"/>
-      <x:c r="K3" s="1"/>
-      <x:c r="L3" s="1"/>
+      <x:c r="B3" s="17"/>
+      <x:c r="C3" s="17"/>
+      <x:c r="D3" s="17"/>
+      <x:c r="E3" s="17"/>
+      <x:c r="F3" s="17"/>
+      <x:c r="G3" s="17"/>
+      <x:c r="H3" s="17"/>
+      <x:c r="I3" s="17"/>
+      <x:c r="J3" s="17"/>
+      <x:c r="K3" s="17"/>
+      <x:c r="L3" s="17"/>
       <x:c r="M3" s="1"/>
       <x:c r="N3" s="1"/>
       <x:c r="O3" s="1"/>
@@ -627,18 +752,18 @@
       <x:c r="R3" s="1"/>
     </x:row>
     <x:row r="4" ht="23" customHeight="1">
-      <x:c r="A4" s="1"/>
-      <x:c r="B4" s="1"/>
-      <x:c r="C4" s="1"/>
-      <x:c r="D4" s="1"/>
-      <x:c r="E4" s="1"/>
-      <x:c r="F4" s="1"/>
-      <x:c r="G4" s="1"/>
-      <x:c r="H4" s="1"/>
-      <x:c r="I4" s="1"/>
-      <x:c r="J4" s="1"/>
-      <x:c r="K4" s="1"/>
-      <x:c r="L4" s="1"/>
+      <x:c r="A4" s="11"/>
+      <x:c r="B4" s="11"/>
+      <x:c r="C4" s="11"/>
+      <x:c r="D4" s="11"/>
+      <x:c r="E4" s="11"/>
+      <x:c r="F4" s="11"/>
+      <x:c r="G4" s="11"/>
+      <x:c r="H4" s="11"/>
+      <x:c r="I4" s="11"/>
+      <x:c r="J4" s="11"/>
+      <x:c r="K4" s="11"/>
+      <x:c r="L4" s="11"/>
       <x:c r="M4" s="1"/>
       <x:c r="N4" s="1"/>
       <x:c r="O4" s="1"/>
@@ -646,23 +771,23 @@
       <x:c r="Q4" s="1"/>
       <x:c r="R4" s="1"/>
     </x:row>
-    <x:row r="5" ht="38" customHeight="1">
-      <x:c r="A5" s="5" t="str">
+    <x:row r="5" ht="27" customHeight="1">
+      <x:c r="A5" s="20" t="str">
         <x:v>Metric</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
+      <x:c r="B5" s="20" t="str">
         <x:v>Value</x:v>
       </x:c>
-      <x:c r="C5" s="1"/>
-      <x:c r="D5" s="1"/>
-      <x:c r="E5" s="1"/>
-      <x:c r="F5" s="1"/>
-      <x:c r="G5" s="1"/>
-      <x:c r="H5" s="1"/>
-      <x:c r="I5" s="1"/>
-      <x:c r="J5" s="1"/>
-      <x:c r="K5" s="1"/>
-      <x:c r="L5" s="1"/>
+      <x:c r="C5" s="11"/>
+      <x:c r="D5" s="11"/>
+      <x:c r="E5" s="11"/>
+      <x:c r="F5" s="11"/>
+      <x:c r="G5" s="11"/>
+      <x:c r="H5" s="11"/>
+      <x:c r="I5" s="11"/>
+      <x:c r="J5" s="11"/>
+      <x:c r="K5" s="11"/>
+      <x:c r="L5" s="11"/>
       <x:c r="M5" s="1"/>
       <x:c r="N5" s="1"/>
       <x:c r="O5" s="1"/>
@@ -670,24 +795,24 @@
       <x:c r="Q5" s="1"/>
       <x:c r="R5" s="1"/>
     </x:row>
-    <x:row r="6" ht="23" customHeight="1">
-      <x:c r="A6" s="1" t="str">
+    <x:row r="6" ht="27" customHeight="1">
+      <x:c r="A6" s="11" t="str">
         <x:v>Inventory value</x:v>
       </x:c>
-      <x:c r="B6" s="6" t="n">
+      <x:c r="B6" s="21" t="n">
         <x:f>SUM('Reorder analysis'!L6:L85)</x:f>
         <x:v>2184017.5499999993</x:v>
       </x:c>
-      <x:c r="C6" s="1"/>
-      <x:c r="D6" s="1"/>
-      <x:c r="E6" s="1"/>
-      <x:c r="F6" s="1"/>
-      <x:c r="G6" s="1"/>
-      <x:c r="H6" s="1"/>
-      <x:c r="I6" s="1"/>
-      <x:c r="J6" s="1"/>
-      <x:c r="K6" s="1"/>
-      <x:c r="L6" s="1"/>
+      <x:c r="C6" s="11"/>
+      <x:c r="D6" s="11"/>
+      <x:c r="E6" s="11"/>
+      <x:c r="F6" s="11"/>
+      <x:c r="G6" s="11"/>
+      <x:c r="H6" s="11"/>
+      <x:c r="I6" s="11"/>
+      <x:c r="J6" s="11"/>
+      <x:c r="K6" s="11"/>
+      <x:c r="L6" s="11"/>
       <x:c r="M6" s="1"/>
       <x:c r="N6" s="1"/>
       <x:c r="O6" s="1"/>
@@ -695,24 +820,24 @@
       <x:c r="Q6" s="1"/>
       <x:c r="R6" s="1"/>
     </x:row>
-    <x:row r="7" ht="23" customHeight="1">
-      <x:c r="A7" s="1" t="str">
+    <x:row r="7" ht="27" customHeight="1">
+      <x:c r="A7" s="11" t="str">
         <x:v>Items requiring reorder</x:v>
       </x:c>
-      <x:c r="B7" s="1" t="n">
+      <x:c r="B7" s="22" t="n">
         <x:f>COUNTIFS('Reorder analysis'!N6:N85,"&gt;0")</x:f>
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C7" s="1"/>
-      <x:c r="D7" s="1"/>
-      <x:c r="E7" s="1"/>
-      <x:c r="F7" s="1"/>
-      <x:c r="G7" s="1"/>
-      <x:c r="H7" s="1"/>
-      <x:c r="I7" s="1"/>
-      <x:c r="J7" s="1"/>
-      <x:c r="K7" s="1"/>
-      <x:c r="L7" s="1"/>
+      <x:c r="C7" s="11"/>
+      <x:c r="D7" s="11"/>
+      <x:c r="E7" s="11"/>
+      <x:c r="F7" s="11"/>
+      <x:c r="G7" s="11"/>
+      <x:c r="H7" s="11"/>
+      <x:c r="I7" s="11"/>
+      <x:c r="J7" s="11"/>
+      <x:c r="K7" s="11"/>
+      <x:c r="L7" s="11"/>
       <x:c r="M7" s="1"/>
       <x:c r="N7" s="1"/>
       <x:c r="O7" s="1"/>
@@ -720,24 +845,24 @@
       <x:c r="Q7" s="1"/>
       <x:c r="R7" s="1"/>
     </x:row>
-    <x:row r="8" ht="23" customHeight="1">
-      <x:c r="A8" s="1" t="str">
+    <x:row r="8" ht="27" customHeight="1">
+      <x:c r="A8" s="11" t="str">
         <x:v>Proposed order cost</x:v>
       </x:c>
-      <x:c r="B8" s="6" t="n">
+      <x:c r="B8" s="21" t="n">
         <x:f>SUM('Reorder analysis'!O6:O85)</x:f>
         <x:v>766792.11</x:v>
       </x:c>
-      <x:c r="C8" s="1"/>
-      <x:c r="D8" s="1"/>
-      <x:c r="E8" s="1"/>
-      <x:c r="F8" s="1"/>
-      <x:c r="G8" s="1"/>
-      <x:c r="H8" s="1"/>
-      <x:c r="I8" s="1"/>
-      <x:c r="J8" s="1"/>
-      <x:c r="K8" s="1"/>
-      <x:c r="L8" s="1"/>
+      <x:c r="C8" s="11"/>
+      <x:c r="D8" s="11"/>
+      <x:c r="E8" s="11"/>
+      <x:c r="F8" s="11"/>
+      <x:c r="G8" s="11"/>
+      <x:c r="H8" s="11"/>
+      <x:c r="I8" s="11"/>
+      <x:c r="J8" s="11"/>
+      <x:c r="K8" s="11"/>
+      <x:c r="L8" s="11"/>
       <x:c r="M8" s="1"/>
       <x:c r="N8" s="1"/>
       <x:c r="O8" s="1"/>
@@ -745,24 +870,24 @@
       <x:c r="Q8" s="1"/>
       <x:c r="R8" s="1"/>
     </x:row>
-    <x:row r="9" ht="23" customHeight="1">
-      <x:c r="A9" s="1" t="str">
+    <x:row r="9" ht="27" customHeight="1">
+      <x:c r="A9" s="11" t="str">
         <x:v>Annualised turnover</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="n">
+      <x:c r="B9" s="23" t="n">
         <x:f>SUM('Reorder analysis'!P6:P85)/SUM('Reorder analysis'!Q6:Q85)*365/90</x:f>
         <x:v>12.42980579869724</x:v>
       </x:c>
-      <x:c r="C9" s="1"/>
-      <x:c r="D9" s="1"/>
-      <x:c r="E9" s="1"/>
-      <x:c r="F9" s="1"/>
-      <x:c r="G9" s="1"/>
-      <x:c r="H9" s="1"/>
-      <x:c r="I9" s="1"/>
-      <x:c r="J9" s="1"/>
-      <x:c r="K9" s="1"/>
-      <x:c r="L9" s="1"/>
+      <x:c r="C9" s="11"/>
+      <x:c r="D9" s="11"/>
+      <x:c r="E9" s="11"/>
+      <x:c r="F9" s="11"/>
+      <x:c r="G9" s="11"/>
+      <x:c r="H9" s="11"/>
+      <x:c r="I9" s="11"/>
+      <x:c r="J9" s="11"/>
+      <x:c r="K9" s="11"/>
+      <x:c r="L9" s="11"/>
       <x:c r="M9" s="1"/>
       <x:c r="N9" s="1"/>
       <x:c r="O9" s="1"/>
@@ -771,18 +896,18 @@
       <x:c r="R9" s="1"/>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
-      <x:c r="A10" s="1"/>
-      <x:c r="B10" s="1"/>
-      <x:c r="C10" s="1"/>
-      <x:c r="D10" s="1"/>
-      <x:c r="E10" s="1"/>
-      <x:c r="F10" s="1"/>
-      <x:c r="G10" s="1"/>
-      <x:c r="H10" s="1"/>
-      <x:c r="I10" s="1"/>
-      <x:c r="J10" s="1"/>
-      <x:c r="K10" s="1"/>
-      <x:c r="L10" s="1"/>
+      <x:c r="A10" s="11"/>
+      <x:c r="B10" s="11"/>
+      <x:c r="C10" s="11"/>
+      <x:c r="D10" s="11"/>
+      <x:c r="E10" s="11"/>
+      <x:c r="F10" s="11"/>
+      <x:c r="G10" s="11"/>
+      <x:c r="H10" s="11"/>
+      <x:c r="I10" s="11"/>
+      <x:c r="J10" s="11"/>
+      <x:c r="K10" s="11"/>
+      <x:c r="L10" s="11"/>
       <x:c r="M10" s="1"/>
       <x:c r="N10" s="1"/>
       <x:c r="O10" s="1"/>
@@ -791,18 +916,18 @@
       <x:c r="R10" s="1"/>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
-      <x:c r="A11" s="1"/>
-      <x:c r="B11" s="1"/>
-      <x:c r="C11" s="1"/>
-      <x:c r="D11" s="1"/>
-      <x:c r="E11" s="1"/>
-      <x:c r="F11" s="1"/>
-      <x:c r="G11" s="1"/>
-      <x:c r="H11" s="1"/>
-      <x:c r="I11" s="1"/>
-      <x:c r="J11" s="1"/>
-      <x:c r="K11" s="1"/>
-      <x:c r="L11" s="1"/>
+      <x:c r="A11" s="11"/>
+      <x:c r="B11" s="11"/>
+      <x:c r="C11" s="11"/>
+      <x:c r="D11" s="11"/>
+      <x:c r="E11" s="11"/>
+      <x:c r="F11" s="11"/>
+      <x:c r="G11" s="11"/>
+      <x:c r="H11" s="11"/>
+      <x:c r="I11" s="11"/>
+      <x:c r="J11" s="11"/>
+      <x:c r="K11" s="11"/>
+      <x:c r="L11" s="11"/>
       <x:c r="M11" s="1"/>
       <x:c r="N11" s="1"/>
       <x:c r="O11" s="1"/>
@@ -810,25 +935,25 @@
       <x:c r="Q11" s="1"/>
       <x:c r="R11" s="1"/>
     </x:row>
-    <x:row r="12" ht="38" customHeight="1">
-      <x:c r="A12" s="5" t="str">
+    <x:row r="12" ht="26" customHeight="1">
+      <x:c r="A12" s="26" t="str">
         <x:v>Category</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="str">
+      <x:c r="B12" s="26" t="str">
         <x:v>Inventory value</x:v>
       </x:c>
-      <x:c r="C12" s="5" t="str">
+      <x:c r="C12" s="26" t="str">
         <x:v>Order cost</x:v>
       </x:c>
-      <x:c r="D12" s="1"/>
-      <x:c r="E12" s="1"/>
-      <x:c r="F12" s="1"/>
-      <x:c r="G12" s="1"/>
-      <x:c r="H12" s="1"/>
-      <x:c r="I12" s="1"/>
-      <x:c r="J12" s="1"/>
-      <x:c r="K12" s="1"/>
-      <x:c r="L12" s="1"/>
+      <x:c r="D12" s="11"/>
+      <x:c r="E12" s="11"/>
+      <x:c r="F12" s="11"/>
+      <x:c r="G12" s="11"/>
+      <x:c r="H12" s="11"/>
+      <x:c r="I12" s="11"/>
+      <x:c r="J12" s="11"/>
+      <x:c r="K12" s="11"/>
+      <x:c r="L12" s="11"/>
       <x:c r="M12" s="1"/>
       <x:c r="N12" s="1"/>
       <x:c r="O12" s="1"/>
@@ -836,27 +961,27 @@
       <x:c r="Q12" s="1"/>
       <x:c r="R12" s="1"/>
     </x:row>
-    <x:row r="13" ht="23" customHeight="1">
-      <x:c r="A13" s="1" t="str">
+    <x:row r="13" ht="26" customHeight="1">
+      <x:c r="A13" s="11" t="str">
         <x:v>Sinks</x:v>
       </x:c>
-      <x:c r="B13" s="6" t="n">
+      <x:c r="B13" s="14" t="n">
         <x:f>SUMIFS('Reorder analysis'!$L$6:$L$85,'Reorder analysis'!$B$6:$B$85,A13)</x:f>
         <x:v>637519.65</x:v>
       </x:c>
-      <x:c r="C13" s="6" t="n">
+      <x:c r="C13" s="14" t="n">
         <x:f>SUMIFS('Reorder analysis'!$O$6:$O$85,'Reorder analysis'!$B$6:$B$85,A13)</x:f>
         <x:v>290238.83</x:v>
       </x:c>
-      <x:c r="D13" s="1"/>
-      <x:c r="E13" s="1"/>
-      <x:c r="F13" s="1"/>
-      <x:c r="G13" s="1"/>
-      <x:c r="H13" s="1"/>
-      <x:c r="I13" s="1"/>
-      <x:c r="J13" s="1"/>
-      <x:c r="K13" s="1"/>
-      <x:c r="L13" s="1"/>
+      <x:c r="D13" s="11"/>
+      <x:c r="E13" s="11"/>
+      <x:c r="F13" s="11"/>
+      <x:c r="G13" s="11"/>
+      <x:c r="H13" s="11"/>
+      <x:c r="I13" s="11"/>
+      <x:c r="J13" s="11"/>
+      <x:c r="K13" s="11"/>
+      <x:c r="L13" s="11"/>
       <x:c r="M13" s="1"/>
       <x:c r="N13" s="1"/>
       <x:c r="O13" s="1"/>
@@ -864,27 +989,27 @@
       <x:c r="Q13" s="1"/>
       <x:c r="R13" s="1"/>
     </x:row>
-    <x:row r="14" ht="23" customHeight="1">
-      <x:c r="A14" s="1" t="str">
+    <x:row r="14" ht="26" customHeight="1">
+      <x:c r="A14" s="11" t="str">
         <x:v>Taps</x:v>
       </x:c>
-      <x:c r="B14" s="6" t="n">
+      <x:c r="B14" s="14" t="n">
         <x:f>SUMIFS('Reorder analysis'!$L$6:$L$85,'Reorder analysis'!$B$6:$B$85,A14)</x:f>
         <x:v>482834.9600000001</x:v>
       </x:c>
-      <x:c r="C14" s="6" t="n">
+      <x:c r="C14" s="14" t="n">
         <x:f>SUMIFS('Reorder analysis'!$O$6:$O$85,'Reorder analysis'!$B$6:$B$85,A14)</x:f>
         <x:v>87785.3</x:v>
       </x:c>
-      <x:c r="D14" s="1"/>
-      <x:c r="E14" s="1"/>
-      <x:c r="F14" s="1"/>
-      <x:c r="G14" s="1"/>
-      <x:c r="H14" s="1"/>
-      <x:c r="I14" s="1"/>
-      <x:c r="J14" s="1"/>
-      <x:c r="K14" s="1"/>
-      <x:c r="L14" s="1"/>
+      <x:c r="D14" s="11"/>
+      <x:c r="E14" s="11"/>
+      <x:c r="F14" s="11"/>
+      <x:c r="G14" s="11"/>
+      <x:c r="H14" s="11"/>
+      <x:c r="I14" s="11"/>
+      <x:c r="J14" s="11"/>
+      <x:c r="K14" s="11"/>
+      <x:c r="L14" s="11"/>
       <x:c r="M14" s="1"/>
       <x:c r="N14" s="1"/>
       <x:c r="O14" s="1"/>
@@ -892,27 +1017,27 @@
       <x:c r="Q14" s="1"/>
       <x:c r="R14" s="1"/>
     </x:row>
-    <x:row r="15" ht="23" customHeight="1">
-      <x:c r="A15" s="1" t="str">
+    <x:row r="15" ht="26" customHeight="1">
+      <x:c r="A15" s="11" t="str">
         <x:v>Hoods</x:v>
       </x:c>
-      <x:c r="B15" s="6" t="n">
+      <x:c r="B15" s="14" t="n">
         <x:f>SUMIFS('Reorder analysis'!$L$6:$L$85,'Reorder analysis'!$B$6:$B$85,A15)</x:f>
         <x:v>356572.66</x:v>
       </x:c>
-      <x:c r="C15" s="6" t="n">
+      <x:c r="C15" s="14" t="n">
         <x:f>SUMIFS('Reorder analysis'!$O$6:$O$85,'Reorder analysis'!$B$6:$B$85,A15)</x:f>
         <x:v>168553.37</x:v>
       </x:c>
-      <x:c r="D15" s="1"/>
-      <x:c r="E15" s="1"/>
-      <x:c r="F15" s="1"/>
-      <x:c r="G15" s="1"/>
-      <x:c r="H15" s="1"/>
-      <x:c r="I15" s="1"/>
-      <x:c r="J15" s="1"/>
-      <x:c r="K15" s="1"/>
-      <x:c r="L15" s="1"/>
+      <x:c r="D15" s="11"/>
+      <x:c r="E15" s="11"/>
+      <x:c r="F15" s="11"/>
+      <x:c r="G15" s="11"/>
+      <x:c r="H15" s="11"/>
+      <x:c r="I15" s="11"/>
+      <x:c r="J15" s="11"/>
+      <x:c r="K15" s="11"/>
+      <x:c r="L15" s="11"/>
       <x:c r="M15" s="1"/>
       <x:c r="N15" s="1"/>
       <x:c r="O15" s="1"/>
@@ -920,27 +1045,27 @@
       <x:c r="Q15" s="1"/>
       <x:c r="R15" s="1"/>
     </x:row>
-    <x:row r="16" ht="23" customHeight="1">
-      <x:c r="A16" s="1" t="str">
+    <x:row r="16" ht="26" customHeight="1">
+      <x:c r="A16" s="11" t="str">
         <x:v>Accessories</x:v>
       </x:c>
-      <x:c r="B16" s="6" t="n">
+      <x:c r="B16" s="14" t="n">
         <x:f>SUMIFS('Reorder analysis'!$L$6:$L$85,'Reorder analysis'!$B$6:$B$85,A16)</x:f>
         <x:v>707090.2799999999</x:v>
       </x:c>
-      <x:c r="C16" s="6" t="n">
+      <x:c r="C16" s="14" t="n">
         <x:f>SUMIFS('Reorder analysis'!$O$6:$O$85,'Reorder analysis'!$B$6:$B$85,A16)</x:f>
         <x:v>220214.61000000002</x:v>
       </x:c>
-      <x:c r="D16" s="1"/>
-      <x:c r="E16" s="1"/>
-      <x:c r="F16" s="1"/>
-      <x:c r="G16" s="1"/>
-      <x:c r="H16" s="1"/>
-      <x:c r="I16" s="1"/>
-      <x:c r="J16" s="1"/>
-      <x:c r="K16" s="1"/>
-      <x:c r="L16" s="1"/>
+      <x:c r="D16" s="11"/>
+      <x:c r="E16" s="11"/>
+      <x:c r="F16" s="11"/>
+      <x:c r="G16" s="11"/>
+      <x:c r="H16" s="11"/>
+      <x:c r="I16" s="11"/>
+      <x:c r="J16" s="11"/>
+      <x:c r="K16" s="11"/>
+      <x:c r="L16" s="11"/>
       <x:c r="M16" s="1"/>
       <x:c r="N16" s="1"/>
       <x:c r="O16" s="1"/>
@@ -949,18 +1074,18 @@
       <x:c r="R16" s="1"/>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
-      <x:c r="A17" s="1"/>
-      <x:c r="B17" s="1"/>
-      <x:c r="C17" s="1"/>
-      <x:c r="D17" s="1"/>
-      <x:c r="E17" s="1"/>
-      <x:c r="F17" s="1"/>
-      <x:c r="G17" s="1"/>
-      <x:c r="H17" s="1"/>
-      <x:c r="I17" s="1"/>
-      <x:c r="J17" s="1"/>
-      <x:c r="K17" s="1"/>
-      <x:c r="L17" s="1"/>
+      <x:c r="A17" s="11"/>
+      <x:c r="B17" s="11"/>
+      <x:c r="C17" s="11"/>
+      <x:c r="D17" s="11"/>
+      <x:c r="E17" s="11"/>
+      <x:c r="F17" s="11"/>
+      <x:c r="G17" s="11"/>
+      <x:c r="H17" s="11"/>
+      <x:c r="I17" s="11"/>
+      <x:c r="J17" s="11"/>
+      <x:c r="K17" s="11"/>
+      <x:c r="L17" s="11"/>
       <x:c r="M17" s="1"/>
       <x:c r="N17" s="1"/>
       <x:c r="O17" s="1"/>
@@ -969,18 +1094,18 @@
       <x:c r="R17" s="1"/>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
-      <x:c r="A18" s="1"/>
-      <x:c r="B18" s="1"/>
-      <x:c r="C18" s="1"/>
-      <x:c r="D18" s="1"/>
-      <x:c r="E18" s="1"/>
-      <x:c r="F18" s="1"/>
-      <x:c r="G18" s="1"/>
-      <x:c r="H18" s="1"/>
-      <x:c r="I18" s="1"/>
-      <x:c r="J18" s="1"/>
-      <x:c r="K18" s="1"/>
-      <x:c r="L18" s="1"/>
+      <x:c r="A18" s="11"/>
+      <x:c r="B18" s="11"/>
+      <x:c r="C18" s="11"/>
+      <x:c r="D18" s="11"/>
+      <x:c r="E18" s="11"/>
+      <x:c r="F18" s="11"/>
+      <x:c r="G18" s="11"/>
+      <x:c r="H18" s="11"/>
+      <x:c r="I18" s="11"/>
+      <x:c r="J18" s="11"/>
+      <x:c r="K18" s="11"/>
+      <x:c r="L18" s="11"/>
       <x:c r="M18" s="1"/>
       <x:c r="N18" s="1"/>
       <x:c r="O18" s="1"/>
@@ -989,20 +1114,20 @@
       <x:c r="R18" s="1"/>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
-      <x:c r="A19" s="1" t="str">
+      <x:c r="A19" s="27" t="str">
         <x:v>Action: filter Proposed units in Reorder analysis to values above zero.</x:v>
       </x:c>
-      <x:c r="B19" s="1"/>
-      <x:c r="C19" s="1"/>
-      <x:c r="D19" s="1"/>
-      <x:c r="E19" s="1"/>
-      <x:c r="F19" s="1"/>
-      <x:c r="G19" s="1"/>
-      <x:c r="H19" s="1"/>
-      <x:c r="I19" s="1"/>
-      <x:c r="J19" s="1"/>
-      <x:c r="K19" s="1"/>
-      <x:c r="L19" s="1"/>
+      <x:c r="B19" s="27"/>
+      <x:c r="C19" s="27"/>
+      <x:c r="D19" s="27"/>
+      <x:c r="E19" s="27"/>
+      <x:c r="F19" s="27"/>
+      <x:c r="G19" s="27"/>
+      <x:c r="H19" s="27"/>
+      <x:c r="I19" s="27"/>
+      <x:c r="J19" s="27"/>
+      <x:c r="K19" s="27"/>
+      <x:c r="L19" s="27"/>
       <x:c r="M19" s="1"/>
       <x:c r="N19" s="1"/>
       <x:c r="O19" s="1"/>
@@ -1011,18 +1136,18 @@
       <x:c r="R19" s="1"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
-      <x:c r="A20" s="1"/>
-      <x:c r="B20" s="1"/>
-      <x:c r="C20" s="1"/>
-      <x:c r="D20" s="1"/>
-      <x:c r="E20" s="1"/>
-      <x:c r="F20" s="1"/>
-      <x:c r="G20" s="1"/>
-      <x:c r="H20" s="1"/>
-      <x:c r="I20" s="1"/>
-      <x:c r="J20" s="1"/>
-      <x:c r="K20" s="1"/>
-      <x:c r="L20" s="1"/>
+      <x:c r="A20" s="11"/>
+      <x:c r="B20" s="11"/>
+      <x:c r="C20" s="11"/>
+      <x:c r="D20" s="11"/>
+      <x:c r="E20" s="11"/>
+      <x:c r="F20" s="11"/>
+      <x:c r="G20" s="11"/>
+      <x:c r="H20" s="11"/>
+      <x:c r="I20" s="11"/>
+      <x:c r="J20" s="11"/>
+      <x:c r="K20" s="11"/>
+      <x:c r="L20" s="11"/>
       <x:c r="M20" s="1"/>
       <x:c r="N20" s="1"/>
       <x:c r="O20" s="1"/>
@@ -1031,20 +1156,20 @@
       <x:c r="R20" s="1"/>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
-      <x:c r="A21" s="1" t="str">
+      <x:c r="A21" s="17" t="str">
         <x:v>Turnover = 90-day demand cost / average stock value × 365 / 90.</x:v>
       </x:c>
-      <x:c r="B21" s="1"/>
-      <x:c r="C21" s="1"/>
-      <x:c r="D21" s="1"/>
-      <x:c r="E21" s="1"/>
-      <x:c r="F21" s="1"/>
-      <x:c r="G21" s="1"/>
-      <x:c r="H21" s="1"/>
-      <x:c r="I21" s="1"/>
-      <x:c r="J21" s="1"/>
-      <x:c r="K21" s="1"/>
-      <x:c r="L21" s="1"/>
+      <x:c r="B21" s="17"/>
+      <x:c r="C21" s="17"/>
+      <x:c r="D21" s="17"/>
+      <x:c r="E21" s="17"/>
+      <x:c r="F21" s="17"/>
+      <x:c r="G21" s="17"/>
+      <x:c r="H21" s="17"/>
+      <x:c r="I21" s="17"/>
+      <x:c r="J21" s="17"/>
+      <x:c r="K21" s="17"/>
+      <x:c r="L21" s="17"/>
       <x:c r="M21" s="1"/>
       <x:c r="N21" s="1"/>
       <x:c r="O21" s="1"/>
@@ -1053,20 +1178,20 @@
       <x:c r="R21" s="1"/>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
-      <x:c r="A22" s="1" t="str">
+      <x:c r="A22" s="17" t="str">
         <x:v>Demand is assumed fulfilled; seasonality is excluded from annualisation.</x:v>
       </x:c>
-      <x:c r="B22" s="1"/>
-      <x:c r="C22" s="1"/>
-      <x:c r="D22" s="1"/>
-      <x:c r="E22" s="1"/>
-      <x:c r="F22" s="1"/>
-      <x:c r="G22" s="1"/>
-      <x:c r="H22" s="1"/>
-      <x:c r="I22" s="1"/>
-      <x:c r="J22" s="1"/>
-      <x:c r="K22" s="1"/>
-      <x:c r="L22" s="1"/>
+      <x:c r="B22" s="17"/>
+      <x:c r="C22" s="17"/>
+      <x:c r="D22" s="17"/>
+      <x:c r="E22" s="17"/>
+      <x:c r="F22" s="17"/>
+      <x:c r="G22" s="17"/>
+      <x:c r="H22" s="17"/>
+      <x:c r="I22" s="17"/>
+      <x:c r="J22" s="17"/>
+      <x:c r="K22" s="17"/>
+      <x:c r="L22" s="17"/>
       <x:c r="M22" s="1"/>
       <x:c r="N22" s="1"/>
       <x:c r="O22" s="1"/>
@@ -1075,20 +1200,20 @@
       <x:c r="R22" s="1"/>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
-      <x:c r="A23" s="1" t="str">
+      <x:c r="A23" s="17" t="str">
         <x:v>Review receipts and allocations before placing any proposed order.</x:v>
       </x:c>
-      <x:c r="B23" s="1"/>
-      <x:c r="C23" s="1"/>
-      <x:c r="D23" s="1"/>
-      <x:c r="E23" s="1"/>
-      <x:c r="F23" s="1"/>
-      <x:c r="G23" s="1"/>
-      <x:c r="H23" s="1"/>
-      <x:c r="I23" s="1"/>
-      <x:c r="J23" s="1"/>
-      <x:c r="K23" s="1"/>
-      <x:c r="L23" s="1"/>
+      <x:c r="B23" s="17"/>
+      <x:c r="C23" s="17"/>
+      <x:c r="D23" s="17"/>
+      <x:c r="E23" s="17"/>
+      <x:c r="F23" s="17"/>
+      <x:c r="G23" s="17"/>
+      <x:c r="H23" s="17"/>
+      <x:c r="I23" s="17"/>
+      <x:c r="J23" s="17"/>
+      <x:c r="K23" s="17"/>
+      <x:c r="L23" s="17"/>
       <x:c r="M23" s="1"/>
       <x:c r="N23" s="1"/>
       <x:c r="O23" s="1"/>
@@ -1097,18 +1222,18 @@
       <x:c r="R23" s="1"/>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
-      <x:c r="A24" s="1"/>
-      <x:c r="B24" s="1"/>
-      <x:c r="C24" s="1"/>
-      <x:c r="D24" s="1"/>
-      <x:c r="E24" s="1"/>
-      <x:c r="F24" s="1"/>
-      <x:c r="G24" s="1"/>
-      <x:c r="H24" s="1"/>
-      <x:c r="I24" s="1"/>
-      <x:c r="J24" s="1"/>
-      <x:c r="K24" s="1"/>
-      <x:c r="L24" s="1"/>
+      <x:c r="A24" s="11"/>
+      <x:c r="B24" s="11"/>
+      <x:c r="C24" s="11"/>
+      <x:c r="D24" s="11"/>
+      <x:c r="E24" s="11"/>
+      <x:c r="F24" s="11"/>
+      <x:c r="G24" s="11"/>
+      <x:c r="H24" s="11"/>
+      <x:c r="I24" s="11"/>
+      <x:c r="J24" s="11"/>
+      <x:c r="K24" s="11"/>
+      <x:c r="L24" s="11"/>
       <x:c r="M24" s="1"/>
       <x:c r="N24" s="1"/>
       <x:c r="O24" s="1"/>
@@ -1117,18 +1242,18 @@
       <x:c r="R24" s="1"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
-      <x:c r="A25" s="1"/>
-      <x:c r="B25" s="1"/>
-      <x:c r="C25" s="1"/>
-      <x:c r="D25" s="1"/>
-      <x:c r="E25" s="1"/>
-      <x:c r="F25" s="1"/>
-      <x:c r="G25" s="1"/>
-      <x:c r="H25" s="1"/>
-      <x:c r="I25" s="1"/>
-      <x:c r="J25" s="1"/>
-      <x:c r="K25" s="1"/>
-      <x:c r="L25" s="1"/>
+      <x:c r="A25" s="11"/>
+      <x:c r="B25" s="11"/>
+      <x:c r="C25" s="11"/>
+      <x:c r="D25" s="11"/>
+      <x:c r="E25" s="11"/>
+      <x:c r="F25" s="11"/>
+      <x:c r="G25" s="11"/>
+      <x:c r="H25" s="11"/>
+      <x:c r="I25" s="11"/>
+      <x:c r="J25" s="11"/>
+      <x:c r="K25" s="11"/>
+      <x:c r="L25" s="11"/>
       <x:c r="M25" s="1"/>
       <x:c r="N25" s="1"/>
       <x:c r="O25" s="1"/>
@@ -2438,7 +2563,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cbd242713944b05"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R091db6ed79184606"/>
 </x:worksheet>
 </file>
 
@@ -8650,7 +8775,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f586cb49dc041fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cee5f448af64e71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12104,7 +12229,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb97505e2dc944fdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c38a82cfcbc40fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>